<commit_message>
added armcd non empty and reran validation
</commit_message>
<xml_diff>
--- a/rules/CORE-002038/positive/01/data/CORE-002038-positive-01.xlsx
+++ b/rules/CORE-002038/positive/01/data/CORE-002038-positive-01.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rich/Documents/github/core-contributor/rules/NEW-RULE/positive/01/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\els_janssens\CORE\Rule_Authoring\core-contributor\rules\CORE-002038\positive\01\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F80DFE97-3C63-3E40-9955-A22739E13350}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B092EDD-EE0C-408A-B109-C96BF6C41AAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Library" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="126">
   <si>
     <t>Product</t>
   </si>
@@ -398,6 +398,9 @@
   </si>
   <si>
     <t>NOTASSGN</t>
+  </si>
+  <si>
+    <t>015246-076-0003-00069</t>
   </si>
 </sst>
 </file>
@@ -847,9 +850,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -857,7 +860,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -873,9 +876,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -883,7 +886,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
@@ -891,7 +894,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
@@ -907,9 +910,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C5FB3F2-2336-DB4C-868B-58728FF11B3C}">
   <dimension ref="A1:T11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:20" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>10</v>
       </c>
@@ -971,7 +974,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:20" ht="64" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:20" ht="75" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>30</v>
       </c>
@@ -1033,7 +1036,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="3" spans="1:20" ht="16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>50</v>
       </c>
@@ -1095,7 +1098,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" s="4">
         <v>12</v>
       </c>
@@ -1157,7 +1160,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:20" ht="32" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:20" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>52</v>
       </c>
@@ -1209,7 +1212,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="6" spans="1:20" ht="48" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:20" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>52</v>
       </c>
@@ -1261,7 +1264,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="7" spans="1:20" ht="48" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:20" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>52</v>
       </c>
@@ -1313,7 +1316,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="8" spans="1:20" ht="48" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:20" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>52</v>
       </c>
@@ -1365,7 +1368,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="9" spans="1:20" ht="32" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:20" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>52</v>
       </c>
@@ -1403,9 +1406,7 @@
       <c r="M9" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="N9" s="3" t="s">
-        <v>75</v>
-      </c>
+      <c r="N9" s="3"/>
       <c r="O9" s="3" t="s">
         <v>76</v>
       </c>
@@ -1421,7 +1422,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="10" spans="1:20" ht="48" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:20" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>52</v>
       </c>
@@ -1477,7 +1478,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="11" spans="1:20" ht="48" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:20" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>52</v>
       </c>
@@ -1542,9 +1543,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CF3CBD5-8954-0240-8A27-54B91AC7B753}">
   <dimension ref="A1:R7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>10</v>
       </c>
@@ -1600,7 +1601,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="64" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:18" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
         <v>30</v>
       </c>
@@ -1656,7 +1657,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>50</v>
       </c>
@@ -1712,7 +1713,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" s="9">
         <v>50</v>
       </c>
@@ -1768,7 +1769,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:18" ht="32" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:18" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>52</v>
       </c>
@@ -1776,7 +1777,7 @@
         <v>108</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>74</v>
+        <v>125</v>
       </c>
       <c r="D5" s="1">
         <v>1</v>
@@ -1822,7 +1823,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:18" ht="32" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:18" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>52</v>
       </c>
@@ -1872,7 +1873,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:18" ht="32" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:18" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>52</v>
       </c>

</xml_diff>